<commit_message>
kaggle sub optimization notebook
</commit_message>
<xml_diff>
--- a/Code/Jupiter/Connect4/Selected EVAL_PPO_results.xlsx
+++ b/Code/Jupiter/Connect4/Selected EVAL_PPO_results.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" state="visible" r:id="rId3"/>
@@ -2914,7 +2914,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+  <sheetPr filterMode="true">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D31"/>
@@ -2934,7 +2934,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" s="1" customFormat="true" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="40" t="s">
         <v>45</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="40" t="s">
         <v>45</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="40" t="n">
         <v>2004</v>
       </c>
@@ -2976,7 +2976,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>2004</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3018,7 +3018,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3032,7 +3032,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="40" t="n">
         <v>2004</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3130,7 +3130,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>802</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3172,7 +3172,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="13.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3340,7 +3340,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="12.8" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="n">
         <v>2004</v>
       </c>
@@ -3355,7 +3355,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D31"/>
+  <autoFilter ref="A1:D31">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="13"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3568,7 +3574,7 @@
       <c r="C4" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>762</v>
       </c>
     </row>
@@ -3582,7 +3588,7 @@
       <c r="C5" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>761</v>
       </c>
     </row>

</xml_diff>